<commit_message>
MP template: KPI + branch dropdowns; importer skips hidden lists sheet
- marketing-template-bycampaign.xlsx: KPI cell has a dropdown (single
  tokens + common combos; still allows typing custom), Branch column in
  the expenses table has a สาขา dropdown. Options stored in a hidden
  "lists" sheet.
- Importer now skips the hidden "lists" sheet.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/marketing-template-bycampaign.xlsx
+++ b/marketing-template-bycampaign.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Energize Hyrox" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Ginger booth" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="คำอธิบาย" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="lists" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -438,7 +439,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
@@ -674,6 +675,14 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=lists!$A$1:$A$13</formula1>
+    </dataValidation>
+    <dataValidation sqref="D14:D63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=lists!$B$1:$B$2</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -688,7 +697,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
@@ -911,6 +920,14 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=lists!$A$1:$A$13</formula1>
+    </dataValidation>
+    <dataValidation sqref="D15:D64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=lists!$B$1:$B$2</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -939,7 +956,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>• แต่ละแท็บ (sheet) = 1 แคมเปญ</t>
+          <t>• แต่ละแท็บ = 1 แคมเปญ</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -956,31 +973,31 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>กรอกข้อมูลแคมเปญแบบ key | value (Campaign, Objective, Start, End, KPI, ผลต่างๆ, Note)</t>
+          <t>กรอกแบบ key | value (Campaign, Objective, Start, End, KPI, ผลต่างๆ, Note)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>• ตาราง "ค่าใช้จ่าย"</t>
+          <t>• KPI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ใส่ได้หลายบรรทัด: Date, Description, Vendor, Branch, Amount — ระบบจะรวมเป็นค่าใช้จ่ายของแคมเปญให้เอง</t>
+          <t>คลิกช่องแล้วมี dropdown ให้เลือก — เลือกหลายอันได้โดยพิมพ์คั่นด้วย , (เช่น acquire, sales)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>• KPI</t>
+          <t>• ตาราง "ค่าใช้จ่าย"</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>คั่นด้วย , : acquire, redemption, sales, awareness, engagement, leads, trial, influencer (เว้นว่าง=เดาให้)</t>
+          <t>ใส่หลายบรรทัด: Date, Description, Vendor, Branch (dropdown), Amount — ระบบรวมให้เอง</t>
         </is>
       </c>
     </row>
@@ -992,19 +1009,134 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ก็อปแท็บตัวอย่าง แล้วแก้ข้อมูล</t>
+          <t>ก็อปแท็บตัวอย่างแล้วแก้ข้อมูล</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>• แท็บนี้ (คำอธิบาย)</t>
+          <t>• แท็บนี้</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
           <t>ระบบจะข้ามให้ ไม่ถูก import</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>acquire</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>สาขา 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>redemption</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>สาขา 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>awareness</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>leads</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>trial</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>influencer</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>acquire, sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>trial, sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>influencer, sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>awareness, engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>acquire, redemption, sales</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MP per-campaign template: all KPI result fields + KPI explanation tab
- Each campaign tab now lists every KPI result field (prefixed by
  [Acquire]/[Trial]/...); fill only the ones for the chosen KPI.
- KPI cell + Branch column are dropdowns.
- "คำอธิบาย" tab maps each KPI → when to use, which result fields to
  fill, and what the app computes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/marketing-template-bycampaign.xlsx
+++ b/marketing-template-bycampaign.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,7 +37,10 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="13"/>
+      <color rgb="002D7A4F"/>
+    </font>
+    <font>
+      <color rgb="00555555"/>
     </font>
   </fonts>
   <fills count="3">
@@ -65,11 +68,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,11 +439,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
@@ -506,171 +510,259 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>—— ผลลัพธ์ (กรอกเฉพาะ KPI ที่เลือก) ——</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>[Acquire] ลูกค้าใหม่ (New)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>200</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>Target</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>250</t>
-        </is>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>[Acquire] Potential</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>46000</t>
-        </is>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>[Acquire] เป้า (Target)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>250</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>[Redemption] Redeem Base (ฐาน)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>[Redemption] Redeem Count</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>[Trial] ผู้มาชิม (Triers)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>[Trial] ตัวอย่างแจก (Samples)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>[Trial] Leads</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>[Trial] ซื้อทันที (Buyers)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>[Influencer] ผู้ติดตามใหม่ (Followers)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>[Awareness] Reach</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>[Awareness] Impressions</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>[Engagement] Engagement</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>[Engagement] Clicks</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>[Sales] ยอดขาย (Sales ฿)</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>46000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>งานวิ่ง Hyrox</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>ค่าใช้จ่าย (Expenses)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Date (วันที่)</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>Description (รายละเอียด)</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>Vendor (ร้าน/แพลตฟอร์ม)</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>Branch (สาขา)</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>Amount (จำนวน ฿)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>2026-05-02</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>Facebook Ads</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Meta</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>สาขา 1</t>
         </is>
       </c>
-      <c r="E14" t="n">
+      <c r="E26" t="n">
         <v>5000</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>คลิปรีวิว influencer</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>อินฟลู A</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>สาขา 1</t>
         </is>
       </c>
-      <c r="E15" t="n">
+      <c r="E27" t="n">
         <v>7427</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>ป้าย/บูธหน้างาน</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>ร้านป้าย</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>สาขา 1</t>
         </is>
       </c>
-      <c r="E16" t="n">
+      <c r="E28" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -679,7 +771,7 @@
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=lists!$A$1:$A$13</formula1>
     </dataValidation>
-    <dataValidation sqref="D14:D63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D26:D75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=lists!$B$1:$B$2</formula1>
     </dataValidation>
   </dataValidations>
@@ -693,11 +785,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
@@ -764,158 +856,236 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>Triers</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>—— ผลลัพธ์ (กรอกเฉพาะ KPI ที่เลือก) ——</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>Samples</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
-      </c>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>[Acquire] ลูกค้าใหม่ (New)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>Leads</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>[Acquire] Potential</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>Buyers</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>[Acquire] เป้า (Target)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>12000</t>
-        </is>
-      </c>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>[Redemption] Redeem Base (ฐาน)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>[Redemption] Redeem Count</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>[Trial] ผู้มาชิม (Triers)</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>[Trial] ตัวอย่างแจก (Samples)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>[Trial] Leads</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>[Trial] ซื้อทันที (Buyers)</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>[Influencer] ผู้ติดตามใหม่ (Followers)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>[Awareness] Reach</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>[Awareness] Impressions</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>[Engagement] Engagement</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>[Engagement] Clicks</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>[Sales] ยอดขาย (Sales ฿)</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>บูทชิมหน้าห้าง</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>ค่าใช้จ่าย (Expenses)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Date (วันที่)</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>Description (รายละเอียด)</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>Vendor (ร้าน/แพลตฟอร์ม)</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>Branch (สาขา)</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>Amount (จำนวน ฿)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>2026-05-10</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>ค่าเช่าพื้นที่บูธ</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>ห้าง</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>สาขา 2</t>
         </is>
       </c>
-      <c r="E15" t="n">
+      <c r="E26" t="n">
         <v>6000</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>2026-05-10</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>ของชิม + แก้ว</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>Makro</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>สาขา 2</t>
         </is>
       </c>
-      <c r="E16" t="n">
+      <c r="E27" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -924,7 +1094,7 @@
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=lists!$A$1:$A$13</formula1>
     </dataValidation>
-    <dataValidation sqref="D15:D64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D26:D75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=lists!$B$1:$B$2</formula1>
     </dataValidation>
   </dataValidations>
@@ -938,90 +1108,230 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="72" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>วิธีใช้ (1 แท็บ = 1 แคมเปญ)</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr"/>
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>ใช้เมื่อไหร่</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>ช่อง result ที่ต้องกรอก</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>ระบบคำนวณให้</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>• แต่ละแท็บ = 1 แคมเปญ</t>
+          <t>acquire</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ตั้งชื่อแท็บเป็นชื่อแคมเปญ หรือใส่ในช่อง Campaign</t>
+          <t>ได้ลูกค้าใหม่ (ซื้อครั้งแรก)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>[Acquire] New, Potential, Target</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>CPA, % เทียบเป้า</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>• ส่วนบน</t>
+          <t>redemption</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>กรอกแบบ key | value (Campaign, Objective, Start, End, KPI, ผลต่างๆ, Note)</t>
+          <t>ลูกค้าใช้คูปอง/กลับมาซื้อ</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>[Redemption] Redeem Base, Redeem Count</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Redemption %</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>• KPI</t>
+          <t>sales</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>คลิกช่องแล้วมี dropdown ให้เลือก — เลือกหลายอันได้โดยพิมพ์คั่นด้วย , (เช่น acquire, sales)</t>
+          <t>วัดยอดขายจากแคมเปญ</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>[Sales] Sales</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ROAS = ยอดขาย ÷ ต้นทุน</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>• ตาราง "ค่าใช้จ่าย"</t>
+          <t>awareness</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ใส่หลายบรรทัด: Date, Description, Vendor, Branch (dropdown), Amount — ระบบรวมให้เอง</t>
+          <t>ทำให้คนรู้จัก (เห็น/เข้าถึง)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>[Awareness] Reach, Impressions</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>CPM</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>• เพิ่มแคมเปญ</t>
+          <t>engagement</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ก็อปแท็บตัวอย่างแล้วแก้ข้อมูล</t>
+          <t>คน interact (ไลก์/คอมเมนต์/คลิก)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>[Engagement] Engagement, Clicks</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>CPE</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>• แท็บนี้</t>
+          <t>leads</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ระบบจะข้ามให้ ไม่ถูก import</t>
+          <t>ได้รายชื่อ/คนสนใจ</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>[Trial] Leads</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>CPL</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>trial</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>บูทชิม/ให้ทดลอง</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>[Trial] Triers, Samples, Leads, Buyers</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>% ชิมแล้วซื้อ, % เป็น lead, ต้นทุน/คนชิม</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>influencer</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>จ้างอินฟลู (ฟอลโลเวอร์)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>[Influencer] Followers + Reach, Engagement, [Sales] Sales</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ต้นทุน/ฟอล, Eng. rate, ROAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>หมายเหตุ</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>เลือก KPI ได้หลายอัน — กรอกเฉพาะช่อง result ของ KPI ที่เลือก ที่เหลือเว้นว่างได้</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ค่าใช้จ่ายใส่เป็นรายการย่อยในตาราง "ค่าใช้จ่าย" ระบบจะรวมเป็นยอดของแคมเปญให้เอง</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MP import: skip Template/ตัวอย่าง sheets; template gets a Template master tab
- Importer now also skips sheets named Template / ตัวอย่าง / แม่แบบ so a
  master tab in the workbook isn't imported as a duplicate campaign.
- marketing-template-bycampaign.xlsx: add a blank "Template" master tab
  (copy to create a new campaign) with KPI + branch dropdowns and all
  result fields; keeps Energize/Ginger examples + คำอธิบาย.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/marketing-template-bycampaign.xlsx
+++ b/marketing-template-bycampaign.xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Energize Hyrox" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Ginger booth" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="คำอธิบาย" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="lists" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet name="Template" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Energize Hyrox" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Ginger booth" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="คำอธิบาย" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="lists" sheetId="5" state="hidden" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,10 +35,6 @@
     </font>
     <font>
       <b val="1"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="002D7A4F"/>
     </font>
     <font>
       <color rgb="00555555"/>
@@ -68,11 +65,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -439,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -457,7 +453,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Energize Hyrox</t>
+          <t>(ชื่อแคมเปญ)</t>
         </is>
       </c>
     </row>
@@ -469,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>เพิ่มลูกค้าใหม่ + ยอดขายงานวิ่ง</t>
+          <t>(วัตถุประสงค์)</t>
         </is>
       </c>
     </row>
@@ -479,11 +475,7 @@
           <t>Start</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-05-01</t>
-        </is>
-      </c>
+      <c r="B3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -491,11 +483,7 @@
           <t>End</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
+      <c r="B4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -503,11 +491,7 @@
           <t>KPI</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>acquire, sales</t>
-        </is>
-      </c>
+      <c r="B5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -518,37 +502,31 @@
       <c r="B6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>[Acquire] ลูกค้าใหม่ (New)</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>200</v>
-      </c>
+      <c r="B7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>[Acquire] Potential</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>50</v>
-      </c>
+      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>[Acquire] เป้า (Target)</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>250</v>
-      </c>
+      <c r="B9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>[Redemption] Redeem Base (ฐาน)</t>
         </is>
@@ -556,7 +534,7 @@
       <c r="B10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>[Redemption] Redeem Count</t>
         </is>
@@ -564,7 +542,7 @@
       <c r="B11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>[Trial] ผู้มาชิม (Triers)</t>
         </is>
@@ -572,7 +550,7 @@
       <c r="B12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>[Trial] ตัวอย่างแจก (Samples)</t>
         </is>
@@ -580,7 +558,7 @@
       <c r="B13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>[Trial] Leads</t>
         </is>
@@ -588,7 +566,7 @@
       <c r="B14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>[Trial] ซื้อทันที (Buyers)</t>
         </is>
@@ -596,7 +574,7 @@
       <c r="B15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>[Influencer] ผู้ติดตามใหม่ (Followers)</t>
         </is>
@@ -604,7 +582,7 @@
       <c r="B16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>[Awareness] Reach</t>
         </is>
@@ -612,7 +590,7 @@
       <c r="B17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>[Awareness] Impressions</t>
         </is>
@@ -620,7 +598,7 @@
       <c r="B18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>[Engagement] Engagement</t>
         </is>
@@ -628,7 +606,7 @@
       <c r="B19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>[Engagement] Clicks</t>
         </is>
@@ -636,14 +614,12 @@
       <c r="B20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>[Sales] ยอดขาย (Sales ฿)</t>
         </is>
       </c>
-      <c r="B21" t="n">
-        <v>46000</v>
-      </c>
+      <c r="B21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
@@ -651,11 +627,7 @@
           <t>Note</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>งานวิ่ง Hyrox</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -665,113 +637,126 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>Date (วันที่)</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Description (รายละเอียด)</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>Vendor (ร้าน/แพลตฟอร์ม)</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>Branch (สาขา)</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>Amount (จำนวน ฿)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>2026-05-02</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Facebook Ads</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>สาขา 1</t>
         </is>
       </c>
-      <c r="E26" t="n">
-        <v>5000</v>
-      </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>คลิปรีวิว influencer</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>อินฟลู A</t>
-        </is>
-      </c>
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
           <t>สาขา 1</t>
         </is>
       </c>
-      <c r="E27" t="n">
-        <v>7427</v>
-      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>ป้าย/บูธหน้างาน</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>ร้านป้าย</t>
-        </is>
-      </c>
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>สาขา 1</t>
         </is>
       </c>
-      <c r="E28" t="n">
-        <v>2000</v>
-      </c>
+      <c r="E28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>สาขา 1</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>สาขา 1</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>สาขา 1</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>สาขา 1</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>สาขา 1</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=lists!$A$1:$A$13</formula1>
     </dataValidation>
-    <dataValidation sqref="D26:D75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D26:D56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=lists!$B$1:$B$2</formula1>
     </dataValidation>
   </dataValidations>
@@ -785,7 +770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -803,7 +788,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Ginger shot sampling booth</t>
+          <t>Energize Hyrox</t>
         </is>
       </c>
     </row>
@@ -815,7 +800,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ให้คนได้ลองชิม เก็บ lead</t>
+          <t>เพิ่มลูกค้าใหม่ + ยอดขายงานวิ่ง</t>
         </is>
       </c>
     </row>
@@ -827,7 +812,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -839,7 +824,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-15</t>
         </is>
       </c>
     </row>
@@ -851,7 +836,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>trial</t>
+          <t>acquire, sales</t>
         </is>
       </c>
     </row>
@@ -864,31 +849,37 @@
       <c r="B6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>[Acquire] ลูกค้าใหม่ (New)</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" t="n">
+        <v>200</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>[Acquire] Potential</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
+      <c r="B8" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>[Acquire] เป้า (Target)</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="n">
+        <v>250</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>[Redemption] Redeem Base (ฐาน)</t>
         </is>
@@ -896,7 +887,7 @@
       <c r="B10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>[Redemption] Redeem Count</t>
         </is>
@@ -904,47 +895,39 @@
       <c r="B11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>[Trial] ผู้มาชิม (Triers)</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>500</v>
-      </c>
+      <c r="B12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>[Trial] ตัวอย่างแจก (Samples)</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>500</v>
-      </c>
+      <c r="B13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>[Trial] Leads</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>80</v>
-      </c>
+      <c r="B14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>[Trial] ซื้อทันที (Buyers)</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>40</v>
-      </c>
+      <c r="B15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>[Influencer] ผู้ติดตามใหม่ (Followers)</t>
         </is>
@@ -952,7 +935,7 @@
       <c r="B16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>[Awareness] Reach</t>
         </is>
@@ -960,7 +943,7 @@
       <c r="B17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>[Awareness] Impressions</t>
         </is>
@@ -968,7 +951,7 @@
       <c r="B18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>[Engagement] Engagement</t>
         </is>
@@ -976,7 +959,7 @@
       <c r="B19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>[Engagement] Clicks</t>
         </is>
@@ -984,13 +967,13 @@
       <c r="B20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>[Sales] ยอดขาย (Sales ฿)</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>12000</v>
+        <v>46000</v>
       </c>
     </row>
     <row r="22">
@@ -999,11 +982,7 @@
           <t>Note</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>บูทชิมหน้าห้าง</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1013,27 +992,27 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>Date (วันที่)</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Description (รายละเอียด)</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>Vendor (ร้าน/แพลตฟอร์ม)</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>Branch (สาขา)</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>Amount (จำนวน ฿)</t>
         </is>
@@ -1042,59 +1021,139 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ค่าเช่าพื้นที่บูธ</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ห้าง</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>สาขา 2</t>
+          <t>สาขา 1</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>6000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ของชิม + แก้ว</t>
+          <t>คลิปรีวิว influencer</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Makro</t>
+          <t>อินฟลู A</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>สาขา 2</t>
+          <t>สาขา 1</t>
         </is>
       </c>
       <c r="E27" t="n">
+        <v>7427</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ป้าย/บูธหน้างาน</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ร้านป้าย</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>สาขา 1</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
         <v>2000</v>
       </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>สาขา 1</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>สาขา 1</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>สาขา 1</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>สาขา 1</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>สาขา 1</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=lists!$A$1:$A$13</formula1>
     </dataValidation>
-    <dataValidation sqref="D26:D75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D26:D56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=lists!$B$1:$B$2</formula1>
     </dataValidation>
   </dataValidations>
@@ -1108,234 +1167,381 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Ginger shot sampling booth</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Objective</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ให้คนได้ลองชิม เก็บ lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>End</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>KPI</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>ใช้เมื่อไหร่</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>ช่อง result ที่ต้องกรอก</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>ระบบคำนวณให้</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>acquire</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>ได้ลูกค้าใหม่ (ซื้อครั้งแรก)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>[Acquire] New, Potential, Target</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>CPA, % เทียบเป้า</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>redemption</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ลูกค้าใช้คูปอง/กลับมาซื้อ</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>[Redemption] Redeem Base, Redeem Count</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Redemption %</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>sales</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>วัดยอดขายจากแคมเปญ</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>[Sales] Sales</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>ROAS = ยอดขาย ÷ ต้นทุน</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>awareness</t>
-        </is>
-      </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ทำให้คนรู้จัก (เห็น/เข้าถึง)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>[Awareness] Reach, Impressions</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>CPM</t>
+          <t>trial</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>engagement</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>คน interact (ไลก์/คอมเมนต์/คลิก)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>[Engagement] Engagement, Clicks</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>CPE</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>—— ผลลัพธ์ (กรอกเฉพาะ KPI ที่เลือก) ——</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>leads</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>ได้รายชื่อ/คนสนใจ</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>[Acquire] ลูกค้าใหม่ (New)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>[Acquire] Potential</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>[Acquire] เป้า (Target)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>[Redemption] Redeem Base (ฐาน)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>[Redemption] Redeem Count</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>[Trial] ผู้มาชิม (Triers)</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>[Trial] ตัวอย่างแจก (Samples)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>[Trial] Leads</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>CPL</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>trial</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>บูทชิม/ให้ทดลอง</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>[Trial] Triers, Samples, Leads, Buyers</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>% ชิมแล้วซื้อ, % เป็น lead, ต้นทุน/คนชิม</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>influencer</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>จ้างอินฟลู (ฟอลโลเวอร์)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>[Influencer] Followers + Reach, Engagement, [Sales] Sales</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>ต้นทุน/ฟอล, Eng. rate, ROAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>หมายเหตุ</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>เลือก KPI ได้หลายอัน — กรอกเฉพาะช่อง result ของ KPI ที่เลือก ที่เหลือเว้นว่างได้</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>ค่าใช้จ่ายใส่เป็นรายการย่อยในตาราง "ค่าใช้จ่าย" ระบบจะรวมเป็นยอดของแคมเปญให้เอง</t>
-        </is>
-      </c>
+      <c r="B14" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>[Trial] ซื้อทันที (Buyers)</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>[Influencer] ผู้ติดตามใหม่ (Followers)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>[Awareness] Reach</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>[Awareness] Impressions</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>[Engagement] Engagement</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>[Engagement] Clicks</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>[Sales] ยอดขาย (Sales ฿)</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ค่าใช้จ่าย (Expenses)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Date (วันที่)</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Description (รายละเอียด)</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Vendor (ร้าน/แพลตฟอร์ม)</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Branch (สาขา)</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Amount (จำนวน ฿)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ค่าเช่าพื้นที่บูธ</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ห้าง</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>สาขา 2</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ของชิม + แก้ว</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>สาขา 2</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>สาขา 1</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>สาขา 1</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>สาขา 1</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>สาขา 1</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>สาขา 1</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>สาขา 1</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=lists!$A$1:$A$13</formula1>
+    </dataValidation>
+    <dataValidation sqref="D26:D56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=lists!$B$1:$B$2</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1346,6 +1552,237 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>ใช้เมื่อไหร่</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>ช่อง result ที่ต้องกรอก</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>ระบบคำนวณให้</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>acquire</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ได้ลูกค้าใหม่ (ซื้อครั้งแรก)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>[Acquire] New, Potential, Target</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>CPA, % เทียบเป้า</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>redemption</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ลูกค้าใช้คูปอง/กลับมาซื้อ</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>[Redemption] Redeem Base, Redeem Count</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Redemption %</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>วัดยอดขายจากแคมเปญ</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>[Sales] Sales</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ROAS = ยอดขาย ÷ ต้นทุน</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>awareness</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ทำให้คนรู้จัก (เห็น/เข้าถึง)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>[Awareness] Reach, Impressions</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>CPM</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>คน interact</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>[Engagement] Engagement, Clicks</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>CPE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>leads</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ได้รายชื่อ/คนสนใจ</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>[Trial] Leads</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>CPL</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>trial</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>บูทชิม/ให้ทดลอง</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>[Trial] Triers, Samples, Leads, Buyers</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>% ชิมแล้วซื้อ, ต้นทุน/คนชิม</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>influencer</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>จ้างอินฟลู (ฟอลโลเวอร์)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>[Influencer] Followers, Reach, Engagement, Sales</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ต้นทุน/ฟอล, ROAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>หมายเหตุ</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ชีต "Template" คือแม่แบบ — ก็อปแล้วเปลี่ยนชื่อแท็บเป็นชื่อแคมเปญ; ระบบจะข้ามชีต Template/คำอธิบาย/lists ตอน import</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>